<commit_message>
Informe y planillas actualizados
</commit_message>
<xml_diff>
--- a/PRINCIPAL/04_Web/archivos/Planillas_Carpinteria_Vortex.xlsx
+++ b/PRINCIPAL/04_Web/archivos/Planillas_Carpinteria_Vortex.xlsx
@@ -15,7 +15,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="291" uniqueCount="139">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="297" uniqueCount="141">
   <si>
     <t>Iluminación de uso general (IUG) — 220 V</t>
   </si>
@@ -323,6 +323,12 @@
     <t>Termomagnético 2P 16 A curva C (TUG1, TUG2, TUG3 y TUE1)</t>
   </si>
   <si>
+    <t>Termomagnético 4P 10 A curva C (salida a los tableros de la lijadora y el compresor 1)</t>
+  </si>
+  <si>
+    <t>Termomagnético 4P 16 A curva C (salida a los tableros de combinada, escuadradora, tupí y sierra sin fin)</t>
+  </si>
+  <si>
     <t>Seccionador bajo carga 4P 100 A</t>
   </si>
   <si>
@@ -335,10 +341,10 @@
     <t>Maniobra</t>
   </si>
   <si>
-    <t>Guardamotor 6–10 A (lijadora, combinada, escuadradora, tupí y sierra sin fin)</t>
-  </si>
-  <si>
-    <t>Guardamotor 4–6,3 A (compresor 1)</t>
+    <t>Guardamotor 6–10 A, en el tablero de cada máquina (lijadora, combinada, escuadradora, tupí y sierra sin fin)</t>
+  </si>
+  <si>
+    <t>Guardamotor 4–6,3 A, en el tablero del compresor 1</t>
   </si>
   <si>
     <t>Contactor 9 A AC-3 bobina 220 V (uno por máquina)</t>
@@ -1512,7 +1518,7 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:F60"/>
+  <dimension ref="A1:F62"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="18" customWidth="1"/>
@@ -2109,14 +2115,14 @@
         <v>84</v>
       </c>
       <c r="D30" s="3">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E30" s="15">
-        <v>70</v>
+        <v>38</v>
       </c>
       <c r="F30" s="15">
         <f>D30*E30</f>
-        <v>70</v>
+        <v>76</v>
       </c>
     </row>
     <row r="31" spans="1:6" x14ac:dyDescent="0.25">
@@ -2130,14 +2136,14 @@
         <v>84</v>
       </c>
       <c r="D31" s="6">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="E31" s="16">
-        <v>11</v>
+        <v>38</v>
       </c>
       <c r="F31" s="16">
         <f>D31*E31</f>
-        <v>11</v>
+        <v>152</v>
       </c>
     </row>
     <row r="32" spans="1:6" x14ac:dyDescent="0.25">
@@ -2154,40 +2160,40 @@
         <v>1</v>
       </c>
       <c r="E32" s="15">
-        <v>60</v>
+        <v>70</v>
       </c>
       <c r="F32" s="15">
         <f>D32*E32</f>
-        <v>60</v>
+        <v>70</v>
       </c>
     </row>
     <row r="33" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A33" s="6" t="s">
+        <v>94</v>
+      </c>
+      <c r="B33" s="6" t="s">
         <v>105</v>
       </c>
-      <c r="B33" s="6" t="s">
-        <v>106</v>
-      </c>
       <c r="C33" s="6" t="s">
         <v>84</v>
       </c>
       <c r="D33" s="6">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="E33" s="16">
-        <v>55</v>
+        <v>11</v>
       </c>
       <c r="F33" s="16">
         <f>D33*E33</f>
-        <v>275</v>
+        <v>11</v>
       </c>
     </row>
     <row r="34" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A34" s="3" t="s">
-        <v>105</v>
+        <v>94</v>
       </c>
       <c r="B34" s="3" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="C34" s="3" t="s">
         <v>84</v>
@@ -2196,16 +2202,16 @@
         <v>1</v>
       </c>
       <c r="E34" s="15">
-        <v>52</v>
+        <v>60</v>
       </c>
       <c r="F34" s="15">
         <f>D34*E34</f>
-        <v>52</v>
+        <v>60</v>
       </c>
     </row>
     <row r="35" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A35" s="6" t="s">
-        <v>105</v>
+        <v>107</v>
       </c>
       <c r="B35" s="6" t="s">
         <v>108</v>
@@ -2214,124 +2220,124 @@
         <v>84</v>
       </c>
       <c r="D35" s="6">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="E35" s="16">
-        <v>35</v>
+        <v>55</v>
       </c>
       <c r="F35" s="16">
         <f>D35*E35</f>
-        <v>210</v>
+        <v>275</v>
       </c>
     </row>
     <row r="36" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A36" s="3" t="s">
-        <v>105</v>
+        <v>107</v>
       </c>
       <c r="B36" s="3" t="s">
         <v>109</v>
       </c>
       <c r="C36" s="3" t="s">
-        <v>110</v>
+        <v>84</v>
       </c>
       <c r="D36" s="3">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="E36" s="15">
-        <v>12</v>
+        <v>52</v>
       </c>
       <c r="F36" s="15">
         <f>D36*E36</f>
-        <v>72</v>
+        <v>52</v>
       </c>
     </row>
     <row r="37" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A37" s="6" t="s">
-        <v>105</v>
+        <v>107</v>
       </c>
       <c r="B37" s="6" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="C37" s="6" t="s">
         <v>84</v>
       </c>
       <c r="D37" s="6">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="E37" s="16">
-        <v>14</v>
+        <v>35</v>
       </c>
       <c r="F37" s="16">
         <f>D37*E37</f>
-        <v>112</v>
+        <v>210</v>
       </c>
     </row>
     <row r="38" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A38" s="3" t="s">
-        <v>105</v>
+        <v>107</v>
       </c>
       <c r="B38" s="3" t="s">
+        <v>111</v>
+      </c>
+      <c r="C38" s="3" t="s">
         <v>112</v>
       </c>
-      <c r="C38" s="3" t="s">
-        <v>84</v>
-      </c>
       <c r="D38" s="3">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="E38" s="15">
-        <v>4</v>
+        <v>12</v>
       </c>
       <c r="F38" s="15">
         <f>D38*E38</f>
-        <v>28</v>
+        <v>72</v>
       </c>
     </row>
     <row r="39" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A39" s="6" t="s">
+        <v>107</v>
+      </c>
+      <c r="B39" s="6" t="s">
         <v>113</v>
       </c>
-      <c r="B39" s="6" t="s">
-        <v>114</v>
-      </c>
       <c r="C39" s="6" t="s">
         <v>84</v>
       </c>
       <c r="D39" s="6">
-        <v>4</v>
+        <v>8</v>
       </c>
       <c r="E39" s="16">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="F39" s="16">
         <f>D39*E39</f>
-        <v>48</v>
+        <v>112</v>
       </c>
     </row>
     <row r="40" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A40" s="3" t="s">
-        <v>113</v>
+        <v>107</v>
       </c>
       <c r="B40" s="3" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="C40" s="3" t="s">
         <v>84</v>
       </c>
       <c r="D40" s="3">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="E40" s="15">
-        <v>25</v>
+        <v>4</v>
       </c>
       <c r="F40" s="15">
         <f>D40*E40</f>
-        <v>150</v>
+        <v>28</v>
       </c>
     </row>
     <row r="41" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A41" s="6" t="s">
-        <v>113</v>
+        <v>115</v>
       </c>
       <c r="B41" s="6" t="s">
         <v>116</v>
@@ -2340,19 +2346,19 @@
         <v>84</v>
       </c>
       <c r="D41" s="6">
-        <v>10</v>
+        <v>4</v>
       </c>
       <c r="E41" s="16">
-        <v>9</v>
+        <v>12</v>
       </c>
       <c r="F41" s="16">
         <f>D41*E41</f>
-        <v>90</v>
+        <v>48</v>
       </c>
     </row>
     <row r="42" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A42" s="3" t="s">
-        <v>113</v>
+        <v>115</v>
       </c>
       <c r="B42" s="3" t="s">
         <v>117</v>
@@ -2364,58 +2370,58 @@
         <v>6</v>
       </c>
       <c r="E42" s="15">
-        <v>45</v>
+        <v>25</v>
       </c>
       <c r="F42" s="15">
         <f>D42*E42</f>
-        <v>270</v>
+        <v>150</v>
       </c>
     </row>
     <row r="43" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A43" s="6" t="s">
+        <v>115</v>
+      </c>
+      <c r="B43" s="6" t="s">
         <v>118</v>
       </c>
-      <c r="B43" s="6" t="s">
-        <v>119</v>
-      </c>
       <c r="C43" s="6" t="s">
         <v>84</v>
       </c>
       <c r="D43" s="6">
-        <v>19</v>
+        <v>10</v>
       </c>
       <c r="E43" s="16">
-        <v>55</v>
+        <v>9</v>
       </c>
       <c r="F43" s="16">
         <f>D43*E43</f>
-        <v>1045</v>
+        <v>90</v>
       </c>
     </row>
     <row r="44" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A44" s="3" t="s">
-        <v>118</v>
+        <v>115</v>
       </c>
       <c r="B44" s="3" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="C44" s="3" t="s">
         <v>84</v>
       </c>
       <c r="D44" s="3">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="E44" s="15">
-        <v>20</v>
+        <v>45</v>
       </c>
       <c r="F44" s="15">
         <f>D44*E44</f>
-        <v>140</v>
+        <v>270</v>
       </c>
     </row>
     <row r="45" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A45" s="6" t="s">
-        <v>118</v>
+        <v>120</v>
       </c>
       <c r="B45" s="6" t="s">
         <v>121</v>
@@ -2424,77 +2430,77 @@
         <v>84</v>
       </c>
       <c r="D45" s="6">
-        <v>2</v>
+        <v>19</v>
       </c>
       <c r="E45" s="16">
-        <v>8</v>
+        <v>55</v>
       </c>
       <c r="F45" s="16">
         <f>D45*E45</f>
-        <v>16</v>
+        <v>1045</v>
       </c>
     </row>
     <row r="46" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A46" s="3" t="s">
-        <v>118</v>
+        <v>120</v>
       </c>
       <c r="B46" s="3" t="s">
         <v>122</v>
       </c>
       <c r="C46" s="3" t="s">
-        <v>88</v>
+        <v>84</v>
       </c>
       <c r="D46" s="3">
-        <v>1</v>
+        <v>7</v>
       </c>
       <c r="E46" s="15">
-        <v>60</v>
+        <v>20</v>
       </c>
       <c r="F46" s="15">
         <f>D46*E46</f>
-        <v>60</v>
+        <v>140</v>
       </c>
     </row>
     <row r="47" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A47" s="6" t="s">
+        <v>120</v>
+      </c>
+      <c r="B47" s="6" t="s">
         <v>123</v>
       </c>
-      <c r="B47" s="6" t="s">
-        <v>124</v>
-      </c>
       <c r="C47" s="6" t="s">
         <v>84</v>
       </c>
       <c r="D47" s="6">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E47" s="16">
-        <v>45</v>
+        <v>8</v>
       </c>
       <c r="F47" s="16">
         <f>D47*E47</f>
-        <v>45</v>
+        <v>16</v>
       </c>
     </row>
     <row r="48" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A48" s="3" t="s">
-        <v>125</v>
+        <v>120</v>
       </c>
       <c r="B48" s="3" t="s">
-        <v>126</v>
+        <v>124</v>
       </c>
       <c r="C48" s="3" t="s">
-        <v>84</v>
+        <v>88</v>
       </c>
       <c r="D48" s="3">
         <v>1</v>
       </c>
       <c r="E48" s="15">
-        <v>150</v>
+        <v>60</v>
       </c>
       <c r="F48" s="15">
         <f>D48*E48</f>
-        <v>150</v>
+        <v>60</v>
       </c>
     </row>
     <row r="49" spans="1:6" x14ac:dyDescent="0.25">
@@ -2502,25 +2508,25 @@
         <v>125</v>
       </c>
       <c r="B49" s="6" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="C49" s="6" t="s">
         <v>84</v>
       </c>
       <c r="D49" s="6">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E49" s="16">
-        <v>18</v>
+        <v>45</v>
       </c>
       <c r="F49" s="16">
         <f>D49*E49</f>
-        <v>36</v>
+        <v>45</v>
       </c>
     </row>
     <row r="50" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A50" s="3" t="s">
-        <v>125</v>
+        <v>127</v>
       </c>
       <c r="B50" s="3" t="s">
         <v>128</v>
@@ -2529,19 +2535,19 @@
         <v>84</v>
       </c>
       <c r="D50" s="3">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E50" s="15">
-        <v>60</v>
+        <v>150</v>
       </c>
       <c r="F50" s="15">
         <f>D50*E50</f>
-        <v>120</v>
+        <v>150</v>
       </c>
     </row>
     <row r="51" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A51" s="6" t="s">
-        <v>125</v>
+        <v>127</v>
       </c>
       <c r="B51" s="6" t="s">
         <v>129</v>
@@ -2553,16 +2559,16 @@
         <v>2</v>
       </c>
       <c r="E51" s="16">
-        <v>25</v>
+        <v>18</v>
       </c>
       <c r="F51" s="16">
         <f>D51*E51</f>
-        <v>50</v>
+        <v>36</v>
       </c>
     </row>
     <row r="52" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A52" s="3" t="s">
-        <v>125</v>
+        <v>127</v>
       </c>
       <c r="B52" s="3" t="s">
         <v>130</v>
@@ -2571,96 +2577,98 @@
         <v>84</v>
       </c>
       <c r="D52" s="3">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="E52" s="15">
-        <v>20</v>
+        <v>60</v>
       </c>
       <c r="F52" s="15">
         <f>D52*E52</f>
-        <v>80</v>
+        <v>120</v>
       </c>
     </row>
     <row r="53" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A53" s="6" t="s">
-        <v>125</v>
+        <v>127</v>
       </c>
       <c r="B53" s="6" t="s">
         <v>131</v>
       </c>
       <c r="C53" s="6" t="s">
-        <v>88</v>
+        <v>84</v>
       </c>
       <c r="D53" s="6">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E53" s="16">
-        <v>220</v>
+        <v>25</v>
       </c>
       <c r="F53" s="16">
         <f>D53*E53</f>
-        <v>220</v>
+        <v>50</v>
       </c>
     </row>
     <row r="54" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A54" s="3" t="s">
-        <v>125</v>
+        <v>127</v>
       </c>
       <c r="B54" s="3" t="s">
         <v>132</v>
       </c>
       <c r="C54" s="3" t="s">
-        <v>88</v>
+        <v>84</v>
       </c>
       <c r="D54" s="3">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="E54" s="15">
-        <v>75</v>
+        <v>20</v>
       </c>
       <c r="F54" s="15">
         <f>D54*E54</f>
+        <v>80</v>
+      </c>
+    </row>
+    <row r="55" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A55" s="6" t="s">
+        <v>127</v>
+      </c>
+      <c r="B55" s="6" t="s">
+        <v>133</v>
+      </c>
+      <c r="C55" s="6" t="s">
+        <v>88</v>
+      </c>
+      <c r="D55" s="6">
+        <v>1</v>
+      </c>
+      <c r="E55" s="16">
+        <v>220</v>
+      </c>
+      <c r="F55" s="16">
+        <f>D55*E55</f>
+        <v>220</v>
+      </c>
+    </row>
+    <row r="56" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A56" s="3" t="s">
+        <v>127</v>
+      </c>
+      <c r="B56" s="3" t="s">
+        <v>134</v>
+      </c>
+      <c r="C56" s="3" t="s">
+        <v>88</v>
+      </c>
+      <c r="D56" s="3">
+        <v>1</v>
+      </c>
+      <c r="E56" s="15">
         <v>75</v>
       </c>
-    </row>
-    <row r="55" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A55" s="9" t="s">
-        <v>16</v>
-      </c>
-      <c r="B55" s="9" t="s">
-        <v>133</v>
-      </c>
-      <c r="C55" s="9" t="s">
-        <v>16</v>
-      </c>
-      <c r="D55" s="9" t="s">
-        <v>16</v>
-      </c>
-      <c r="E55" s="17" t="s">
-        <v>16</v>
-      </c>
-      <c r="F55" s="17">
-        <v>6998.8</v>
-      </c>
-    </row>
-    <row r="56" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A56" s="9" t="s">
-        <v>16</v>
-      </c>
-      <c r="B56" s="9" t="s">
-        <v>134</v>
-      </c>
-      <c r="C56" s="9" t="s">
-        <v>16</v>
-      </c>
-      <c r="D56" s="9" t="s">
-        <v>16</v>
-      </c>
-      <c r="E56" s="17" t="s">
-        <v>16</v>
-      </c>
-      <c r="F56" s="17">
-        <v>2449.58</v>
+      <c r="F56" s="15">
+        <f>D56*E56</f>
+        <v>75</v>
       </c>
     </row>
     <row r="57" spans="1:6" x14ac:dyDescent="0.25">
@@ -2680,7 +2688,7 @@
         <v>16</v>
       </c>
       <c r="F57" s="17">
-        <v>699.88</v>
+        <v>7226.8</v>
       </c>
     </row>
     <row r="58" spans="1:6" x14ac:dyDescent="0.25">
@@ -2700,7 +2708,7 @@
         <v>16</v>
       </c>
       <c r="F58" s="17">
-        <v>472.42</v>
+        <v>2529.38</v>
       </c>
     </row>
     <row r="59" spans="1:6" x14ac:dyDescent="0.25">
@@ -2720,7 +2728,7 @@
         <v>16</v>
       </c>
       <c r="F59" s="17">
-        <v>2230.34</v>
+        <v>722.68</v>
       </c>
     </row>
     <row r="60" spans="1:6" x14ac:dyDescent="0.25">
@@ -2740,7 +2748,47 @@
         <v>16</v>
       </c>
       <c r="F60" s="17">
-        <v>12851.02</v>
+        <v>487.81</v>
+      </c>
+    </row>
+    <row r="61" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A61" s="9" t="s">
+        <v>16</v>
+      </c>
+      <c r="B61" s="9" t="s">
+        <v>139</v>
+      </c>
+      <c r="C61" s="9" t="s">
+        <v>16</v>
+      </c>
+      <c r="D61" s="9" t="s">
+        <v>16</v>
+      </c>
+      <c r="E61" s="17" t="s">
+        <v>16</v>
+      </c>
+      <c r="F61" s="17">
+        <v>2303</v>
+      </c>
+    </row>
+    <row r="62" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A62" s="9" t="s">
+        <v>16</v>
+      </c>
+      <c r="B62" s="9" t="s">
+        <v>140</v>
+      </c>
+      <c r="C62" s="9" t="s">
+        <v>16</v>
+      </c>
+      <c r="D62" s="9" t="s">
+        <v>16</v>
+      </c>
+      <c r="E62" s="17" t="s">
+        <v>16</v>
+      </c>
+      <c r="F62" s="17">
+        <v>13269.67</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Unifilar corregido, sin topográficos propios, sección de tableros
</commit_message>
<xml_diff>
--- a/PRINCIPAL/04_Web/archivos/Planillas_Carpinteria_Vortex.xlsx
+++ b/PRINCIPAL/04_Web/archivos/Planillas_Carpinteria_Vortex.xlsx
@@ -323,10 +323,10 @@
     <t>Termomagnético 2P 16 A curva C (TUG1, TUG2, TUG3 y TUE1)</t>
   </si>
   <si>
-    <t>Termomagnético 4P 10 A curva C (salida a los tableros de la lijadora y el compresor 1)</t>
-  </si>
-  <si>
-    <t>Termomagnético 4P 16 A curva C (salida a los tableros de combinada, escuadradora, tupí y sierra sin fin)</t>
+    <t>Termomagnético 4P 10 A curva C (salida al tablero de la lijadora)</t>
+  </si>
+  <si>
+    <t>Termomagnético 4P 16 A curva C (salida a los tableros de combinada, escuadradora, tupí, sierra sin fin y compresor 1)</t>
   </si>
   <si>
     <t>Seccionador bajo carga 4P 100 A</t>
@@ -2115,14 +2115,14 @@
         <v>84</v>
       </c>
       <c r="D30" s="3">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E30" s="15">
         <v>38</v>
       </c>
       <c r="F30" s="15">
         <f>D30*E30</f>
-        <v>76</v>
+        <v>38</v>
       </c>
     </row>
     <row r="31" spans="1:6" x14ac:dyDescent="0.25">
@@ -2136,14 +2136,14 @@
         <v>84</v>
       </c>
       <c r="D31" s="6">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="E31" s="16">
         <v>38</v>
       </c>
       <c r="F31" s="16">
         <f>D31*E31</f>
-        <v>152</v>
+        <v>190</v>
       </c>
     </row>
     <row r="32" spans="1:6" x14ac:dyDescent="0.25">

</xml_diff>